<commit_message>
update interface, ui, process
</commit_message>
<xml_diff>
--- a/SVI_NFT_R/SEQUENCE/Main/00_EqToEq/SDV Gamma Foldable Line/GeneratedSource/DataGroups/EqToEq/EqToEq.BitDeviceMap.xlsx
+++ b/SVI_NFT_R/SEQUENCE/Main/00_EqToEq/SDV Gamma Foldable Line/GeneratedSource/DataGroups/EqToEq/EqToEq.BitDeviceMap.xlsx
@@ -1,31 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\SVI_NFT_R\SVI_NFT_R\SEQUENCE\Main\00_EqToEq\SDV Gamma Foldable Line\GeneratedSource\DataGroups\EqToEq\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\01. ENC\02_Samsung\08_V34F_NFT\01_Program\SVI_NFT_R_Type3_55-60_nguyen\SVI_NFT_R\SVI_NFT_R\SEQUENCE\Main\00_EqToEq\SDV Gamma Foldable Line\GeneratedSource\DataGroups\EqToEq\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0715AF7D-C455-4DFF-AD19-690762E2F6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12285"/>
+    <workbookView xWindow="8415" yWindow="3885" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Map" sheetId="1" r:id="rId1"/>
     <sheet name="Define" sheetId="4" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Description</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -149,24 +161,42 @@
   <si>
     <t>4100</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SelfToLower</t>
+  </si>
+  <si>
+    <t>EqToEq.SelfToLower.Bits</t>
+  </si>
+  <si>
+    <t>시작 비트 주소는 0x3480</t>
+  </si>
+  <si>
+    <t>LowerToSelf</t>
+  </si>
+  <si>
+    <t>EqToEq.LowerToSelf.Bits</t>
+  </si>
+  <si>
+    <t>시작 비트 주소는 0x3700</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -179,9 +209,14 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -214,20 +249,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="표준 12" xfId="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준 12" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -271,20 +307,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="표1_34" displayName="표1_34" ref="A1:I3" totalsRowShown="0">
-  <autoFilter ref="A1:I3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표1_34" displayName="표1_34" ref="A1:I5" totalsRowShown="0">
+  <autoFilter ref="A1:I5" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="9">
-    <tableColumn id="2" name="ID"/>
-    <tableColumn id="13" name="Byte Index(or Offset)" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ID"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Byte Index(or Offset)" dataDxfId="1">
       <calculatedColumnFormula>HEX2DEC(K2)/8</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" name="Bit Index"/>
-    <tableColumn id="7" name="Handling Data Type"/>
-    <tableColumn id="8" name="Array Length"/>
-    <tableColumn id="9" name="Decimal Point"/>
-    <tableColumn id="19" name="Label"/>
-    <tableColumn id="16" name="Description"/>
-    <tableColumn id="17" name="Comment" dataDxfId="0" dataCellStyle="표준 12">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Bit Index"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Handling Data Type"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Array Length"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Decimal Point"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Label"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Description"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Comment" dataDxfId="0" dataCellStyle="표준 12">
       <calculatedColumnFormula>"시작 비트 주소는 0x"&amp;K2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -293,10 +329,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:A15" totalsRowShown="0">
-  <autoFilter ref="A1:A15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="표1" displayName="표1" ref="A1:A15" totalsRowShown="0">
+  <autoFilter ref="A1:A15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="1">
-    <tableColumn id="1" name="데이터 타입"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="데이터 타입"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -564,22 +600,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.875" customWidth="1"/>
-    <col min="2" max="2" width="22.25" customWidth="1"/>
-    <col min="3" max="3" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.375" customWidth="1"/>
-    <col min="5" max="5" width="15.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.375" customWidth="1"/>
-    <col min="9" max="9" width="40.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.42578125" customWidth="1"/>
+    <col min="9" max="9" width="40.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -611,70 +647,106 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2">
         <f>HEX2DEC(K2)/8</f>
         <v>2032</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="2" t="str">
+      <c r="I2" s="1" t="str">
         <f>"시작 비트 주소는 0x"&amp;K2</f>
         <v>시작 비트 주소는 0x3F80</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="1">
-        <f t="shared" ref="B3" si="0">HEX2DEC(K3)/8</f>
+      <c r="B3">
+        <f t="shared" ref="B3:B5" si="0">HEX2DEC(K3)/8</f>
         <v>2080</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="2" t="str">
+      <c r="I3" s="1" t="str">
         <f>"시작 비트 주소는 0x"&amp;K3</f>
         <v>시작 비트 주소는 0x4100</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>1680</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4">
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>1760</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5">
+        <v>3700</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="8">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="배열의 길이" prompt="  해당 파라미터가 공백이면 단일 데이터로 생성하고, 정수 값이 입력되면 배열 데이터로 생성합니다._x000a__x000a_유효 데이터: _x000a_  - 공백 (단일 타입)_x000a_  - 1 ~ 2147483647 (배열 타입)" sqref="E2:E3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="배열의 길이" prompt="  해당 파라미터가 공백이면 단일 데이터로 생성하고, 정수 값이 입력되면 배열 데이터로 생성합니다._x000a__x000a_유효 데이터: _x000a_  - 공백 (단일 타입)_x000a_  - 1 ~ 2147483647 (배열 타입)" sqref="E2:E5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="textLength" imeMode="halfAlpha" showInputMessage="1" showErrorMessage="1" promptTitle="ID (변수명)" prompt="데이터의 고유한 이름을 설정합니다._x000a__x000a_※ID는 코드 변환시 변수명으로 사용되기 때문에 C#문법에서 허용하지 않는 작명 방식은 지원하지 않음" sqref="A2:A3">
+    <dataValidation type="textLength" imeMode="halfAlpha" showInputMessage="1" showErrorMessage="1" promptTitle="ID (변수명)" prompt="데이터의 고유한 이름을 설정합니다._x000a__x000a_※ID는 코드 변환시 변수명으로 사용되기 때문에 C#문법에서 허용하지 않는 작명 방식은 지원하지 않음" sqref="A2:A5" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>1</formula1>
       <formula2>256</formula2>
     </dataValidation>
-    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" promptTitle="바이트 인덱스(or 오프셋)" prompt="  해당 데이터의 위치를 나타내는 정보를 설정합니다._x000a__x000a_유효 데이터:_x000a_- 'auto'_x000a_- 0 ~ 2147483647_x000a__x000a_※ 'auto'란?_x000a_이전 데이터가 끝난 다음 위치를 자동으로 계산해서 넣어주는 기능" sqref="B2:B3">
+    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" promptTitle="바이트 인덱스(or 오프셋)" prompt="  해당 데이터의 위치를 나타내는 정보를 설정합니다._x000a__x000a_유효 데이터:_x000a_- 'auto'_x000a_- 0 ~ 2147483647_x000a__x000a_※ 'auto'란?_x000a_이전 데이터가 끝난 다음 위치를 자동으로 계산해서 넣어주는 기능" sqref="B2:B5" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>IF(ISNUMBER(B2), AND(B2 &gt; 0, B2 &lt; 2147483647), AND(LOWER(B2) = "auto", NOT(ISBLANK(B2))))</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="비트 인덱스" prompt="  해당 데이터의 위치를 나타내는 정보를 설정합니다._x000a__x000a_유효 데이터:_x000a_- 공백 (bool형이 선택되지 않았을 때)_x000a_- 0 ~ 7 (bool형이 선택됐을 때)_x000a__x000a_※'Bit Index'는 'Handling Data Tpye'이 'bool'로 설정됐을 때에만 적용됩니다." sqref="C2:C3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="비트 인덱스" prompt="  해당 데이터의 위치를 나타내는 정보를 설정합니다._x000a__x000a_유효 데이터:_x000a_- 공백 (bool형이 선택되지 않았을 때)_x000a_- 0 ~ 7 (bool형이 선택됐을 때)_x000a__x000a_※'Bit Index'는 'Handling Data Tpye'이 'bool'로 설정됐을 때에만 적용됩니다." sqref="C2:C5" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
       <formula2>7</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="소수점 위치" prompt="(옵션)" sqref="F2:F3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="소수점 위치" prompt="(옵션)" sqref="F2:F5" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="라벨" prompt="(옵션)" sqref="G2:G3"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="코맨트" prompt="(옵션)" sqref="I2:I3"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="설명" prompt="(옵션)" sqref="H2:H3"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="라벨" prompt="(옵션)" sqref="G2:G5" xr:uid="{00000000-0002-0000-0000-000005000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="코맨트" prompt="(옵션)" sqref="I2:I5" xr:uid="{00000000-0002-0000-0000-000006000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="설명" prompt="(옵션)" sqref="H2:H5" xr:uid="{00000000-0002-0000-0000-000007000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -684,11 +756,11 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" imeMode="halfAlpha" showInputMessage="1" promptTitle="데이터 타입" prompt="  해당 데이터의 타입을 설정합니다._x000a__x000a_데이터 범위:_x000a_- 사용자 정의 데이터 블록 타입_x000a_- 기본 데이터 타입(bool, byte, sbyte, ushort, short, uint, int, ulong, long, float, double, char)_x000a_">
+        <x14:dataValidation type="list" imeMode="halfAlpha" showInputMessage="1" promptTitle="데이터 타입" prompt="  해당 데이터의 타입을 설정합니다._x000a__x000a_데이터 범위:_x000a_- 사용자 정의 데이터 블록 타입_x000a_- 기본 데이터 타입(bool, byte, sbyte, ushort, short, uint, int, ulong, long, float, double, char)_x000a_" xr:uid="{00000000-0002-0000-0000-000008000000}">
           <x14:formula1>
             <xm:f>Define!$A$2:$A$15</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D3</xm:sqref>
+          <xm:sqref>D2:D5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -697,87 +769,87 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.75" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1">
       <c r="A8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1">
       <c r="A10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1">
       <c r="A11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1">
       <c r="A12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1">
       <c r="A13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1">
       <c r="A14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1">
       <c r="A15" t="s">
         <v>21</v>
       </c>

</xml_diff>